<commit_message>
Versión 3.8: nueva funcionalidad en pre-sim, pre-equipos y recargas
</commit_message>
<xml_diff>
--- a/src/consulta_seriales/seriales.xlsx
+++ b/src/consulta_seriales/seriales.xlsx
@@ -425,119 +425,722 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:A102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Iccid</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Imei</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Mensaje</t>
+          <t>seriales</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602308230397</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> nan</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>El ICC_ID 89571016023082303973 ESTA EN USO</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602308230411</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> nan</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>El ICC_ID 89571016023082304112 ESTA EN USO</t>
+          <t>201</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> nan</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 867452070086942</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>202</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> nan</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 867452070165589</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>es principal</t>
+          <t>203</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> nan</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 353283531154719</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>204</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602308198896</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> nan</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>205</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>207</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>208</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>216</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>217</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>218</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>219</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>221</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>234</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>237</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>239</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>241</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>242</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>243</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>244</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>245</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>246</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>247</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>248</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>249</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>251</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>252</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>253</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>254</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>257</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>258</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>259</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>261</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>262</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>263</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>264</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>265</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>266</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>267</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>268</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>269</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>270</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>271</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>272</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>273</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>274</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>275</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>277</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>278</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>279</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>280</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>281</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>282</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>283</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>284</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>285</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>286</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>287</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>288</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>289</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>290</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>291</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>292</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>293</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>294</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>295</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>296</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>297</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>298</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>299</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>